<commit_message>
Remove stray total-formula cell from the downloadable sample workbook
Row 5 of the sample sheet had a leftover =SUM(I4:I4) formula in the
Deducted VAT column with every other cell blank -- not part of the
intended example, but enough to make the importer flag it as an
invalid row ("VAT/rate must be greater than 0") the moment someone
downloaded the sample and re-uploaded it as-is. Removed just that
formula cell (and its calcChain entry) directly in the xlsx XML so
the file's other content and size stay untouched.
</commit_message>
<xml_diff>
--- a/frontend/public/Sample_VDS_Format.xlsx
+++ b/frontend/public/Sample_VDS_Format.xlsx
@@ -6245,12 +6245,6 @@
         <v>58</v>
       </c>
     </row>
-    <row r="5" spans="1:13" x14ac:dyDescent="0.4">
-      <c r="I5" s="68">
-        <f>SUM(I4:I4)</f>
-        <v>1085</v>
-      </c>
-    </row>
   </sheetData>
   <autoFilter ref="A3:J3" xr:uid="{00000000-0009-0000-0000-000014000000}">
     <sortState xmlns:xlrd2="http://schemas.microsoft.com/office/spreadsheetml/2017/richdata2" ref="A4:J23">

</xml_diff>